<commit_message>
Reorganise homepage and modify welcome texts
</commit_message>
<xml_diff>
--- a/data-raw/project_texts.xlsx
+++ b/data-raw/project_texts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neilm\Projects\b_useful\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{653D348E-0D0A-4163-9A9F-D6BE72D3CDBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{028E4A9D-2C97-4141-B32A-7361851EFF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
   </bookViews>
@@ -18,6 +18,8 @@
     <sheet name="themes" sheetId="2" r:id="rId3"/>
     <sheet name="case_studies" sheetId="3" r:id="rId4"/>
     <sheet name="fig_text" sheetId="5" r:id="rId5"/>
+    <sheet name="tooltips" sheetId="6" r:id="rId6"/>
+    <sheet name="sources" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="51">
   <si>
     <t>text</t>
   </si>
@@ -56,12 +58,6 @@
   </si>
   <si>
     <t xml:space="preserve">B-USEFUL results were generated by a consortium of 13 partner institutes from 11 countries. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">B-USEFUL aims to contribute to achieve the policy goals set out by the EU Green Deal and the Biodiversity Strategy 2030 by developing user-oriented tools and solutions to conserve marine biodiversity. Learn more more about B-USEFUL in &lt;em&gt;About&lt;/em&gt; or at the  &lt;a href="https://b-useful.eu/"&gt;B-USEFUL project website&lt;/a&gt;. &lt;br&gt;&lt;br&gt;
-&lt;h4&gt; What can I find in this toolbox? &lt;/h4&gt;&lt;p&gt;Lots of recent scientific results from the project, covering multiple dimensions of biodiversity: results are organised by the broad B-USEFUL themes.
-&lt;h4&gt; How do I use this tool? &lt;/h4&gt;&lt;p&gt;&lt;li&gt;Select a case study region of interest from the dropdown or &lt;em&gt;Results&lt;/em&gt; tab of the navbar - you will be directed to the results.&lt;/li&gt;&lt;li&gt;Navigate through the themes of B-USEFUL using the top-level tabs.&lt;/li&gt;&lt;li&gt;Explore particular aspects of these themes with the second level of tabs&lt;/li&gt;&lt;li&gt;Use the controls in the sidebars to filter the outputs according to interest&lt;/li&gt;&lt;li&gt;Learn about Biodiversity in European Seas!&lt;/li&gt;
-</t>
   </si>
   <si>
     <t>intro</t>
@@ -133,6 +129,70 @@
       The interface, organisation and guidance and functionality can be modified to make the DST more useful and accessible, according to your feedback.
 &lt;br&gt;&lt;hr&gt;&lt;h4&gt;Disclaimer: &lt;/h4&gt;
        This tool has not yet been finalised and the data presented will be updated to reflect the final modelling outputs. Data from the DST should not be applied elsewhere prior to the finalisation of the project on 30th September 2026.</t>
+  </si>
+  <si>
+    <t>richness</t>
+  </si>
+  <si>
+    <t>evenness</t>
+  </si>
+  <si>
+    <t>shannon</t>
+  </si>
+  <si>
+    <t>fric</t>
+  </si>
+  <si>
+    <t>feve</t>
+  </si>
+  <si>
+    <t>fdiv</t>
+  </si>
+  <si>
+    <t>fdis</t>
+  </si>
+  <si>
+    <t>Functional evenness indices measure whether mean species traits are distributed regularly within the occupied trait space.</t>
+  </si>
+  <si>
+    <t>Functional Richness measures how much of the niche space is occupied by the species present.</t>
+  </si>
+  <si>
+    <t>functional_diversity_indices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schleuter, Diana &amp; Daufresne, Martin &amp; Massol, François. (2010). A user's guide to functional diversity indices. Ecological Monographs. 80. 469-484. 10.2307/20787442. </t>
+  </si>
+  <si>
+    <t>Functional divergence measures the variance of the species’ functions and the position of their clusters in trait space. High values indicate that the dominant species have extreme traits.</t>
+  </si>
+  <si>
+    <t>Function dispersion measures how far species are, on average, from the community average traits. High values indicate an assemblage where species are generally quite different and where there are many ecological roles.</t>
+  </si>
+  <si>
+    <t>Species Richness is the number of species that are present in a given area.</t>
+  </si>
+  <si>
+    <t>Shannon Index measures the proportional abundance of species in an assemblage. For a given number of species, an assemblage with higher evenness will have a higher shannon index.</t>
+  </si>
+  <si>
+    <t>Relative abundance of different species within a community or ecosystem.</t>
+  </si>
+  <si>
+    <t>what</t>
+  </si>
+  <si>
+    <t>how</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;h4&gt; What can I find in this toolbox? &lt;/h4&gt;&lt;p&gt; Maps, animations and time-series of biodiversity of fish and benthos in Europe, from the Barents Sea to the Central Mediterranean Sea. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-USEFUL aims to contribute to achieve the policy goals set out by the EU Green Deal and the Biodiversity Strategy 2030 by developing user-oriented tools and solutions to conserve marine biodiversity. B-USEFUL applies a consistent methodology to much of Europe's seas to provide a new model infrastructure to better characterize and forecast changes in marine biodiversity. In doing so it generates new understanding of marine biodiversity in Europe. Learn more more about B-USEFUL in &lt;em&gt;About&lt;/em&gt; or at the  &lt;a href="https://b-useful.eu/"&gt;B-USEFUL project website&lt;/a&gt;.
+</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt; How do I use this tool? &lt;/h4&gt;&lt;p&gt;&lt;li&gt;Select a case study region of interest from the dropdown or &lt;em&gt;Results&lt;/em&gt; tab of the navbar - you will be directed to the results.&lt;/li&gt;&lt;li&gt;use the &lt;em&gt;Explore&lt;/em&gt; tab to investigate the historical and projected changes in biodiversity for a range of indicators.&lt;/li&gt;&lt;li&gt;Use the  &lt;em&gt;Interactive tool&lt;/em&gt; tab to identify areas meeting your criteria.&lt;/li&gt;</t>
   </si>
 </sst>
 </file>
@@ -508,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFAC5F67-39A2-465C-88B9-4321F2EB8BB8}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
@@ -524,48 +584,64 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="88.5" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
-      <c r="A6" t="s">
+    <row r="8" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="B7" s="1"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="B9" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -592,63 +668,63 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
         <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="77.45" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
         <v>23</v>
-      </c>
-      <c r="B8" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -762,20 +838,128 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24344193-A5DC-4C09-A7D0-962941565ADB}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <cols>
+    <col min="2" max="2" width="60.2265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52622770-8B11-4F83-8FC4-BE5BFE84B716}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <cols>
+    <col min="1" max="1" width="25.58984375" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tidy up and add new texts to landing page
</commit_message>
<xml_diff>
--- a/data-raw/project_texts.xlsx
+++ b/data-raw/project_texts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neilm\Projects\b_useful\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{028E4A9D-2C97-4141-B32A-7361851EFF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FF5C0F-1624-4EC7-A5E8-F7570D3C0BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="landing_page" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
   <si>
     <t>text</t>
   </si>
@@ -179,20 +179,57 @@
     <t>Relative abundance of different species within a community or ecosystem.</t>
   </si>
   <si>
-    <t>what</t>
+    <t xml:space="preserve">From the Greenland and Barents Seas to the Mediterranean, B-USEFUL aims to contribute to achieve the policy goals set out by the EU Green Deal and the Biodiversity Strategy 2030 by developing user-oriented tools and solutions to conserve marine biodiversity. B-USEFUL applies a consistent methodology across Europe's seas to provide a new model infrastructure to better characterize and forecast changes in marine biodiversity. In doing so it generates new understanding of marine biodiversity in Europe. Learn more more about B-USEFUL in &lt;em&gt;About&lt;/em&gt; or at the  &lt;a href="https://b-useful.eu/"&gt;B-USEFUL project website&lt;/a&gt;.
+</t>
+  </si>
+  <si>
+    <t>what1</t>
+  </si>
+  <si>
+    <t>what2</t>
+  </si>
+  <si>
+    <t>Explore spatial and temporal patterns and changes in fish and demersal biodiversity in Europe, from the Barents Sea to the Eastern Mediterranean Sea: &lt;br&gt;&lt;ul&gt;
+&lt;li&gt;View maps and animations for several taxonomic and functional biodiversity indices. &lt;/li&gt;&lt;br&gt;
+&lt;li&gt;Select and compare side-by-side plots of different year results or see the overall trend through the study period. &lt;/li&gt;&lt;br&gt;
+&lt;li&gt;Get biodiversity summary statistics for user-defined areas.&lt;/li&gt;&lt;/ul&gt;</t>
+  </si>
+  <si>
+    <t>&lt;br&gt;&lt;br&gt;&lt;ul&gt;&lt;li&gt;Filter areas based on biodiversity indices to show areas meeting user-defined biodiversity criteria.&lt;/li&gt;&lt;br&gt;
+&lt;li&gt;Combine spatial and biodiversity filters to identify hotspots within particular areas.&lt;/li&gt;&lt;br&gt;
+&lt;li&gt;In a future version users will be able to overlay biodiversity layers with Human Activity and Pressure layers.&lt;/ul&gt;</t>
   </si>
   <si>
     <t>how</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;h4&gt; What can I find in this toolbox? &lt;/h4&gt;&lt;p&gt; Maps, animations and time-series of biodiversity of fish and benthos in Europe, from the Barents Sea to the Central Mediterranean Sea. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">B-USEFUL aims to contribute to achieve the policy goals set out by the EU Green Deal and the Biodiversity Strategy 2030 by developing user-oriented tools and solutions to conserve marine biodiversity. B-USEFUL applies a consistent methodology to much of Europe's seas to provide a new model infrastructure to better characterize and forecast changes in marine biodiversity. In doing so it generates new understanding of marine biodiversity in Europe. Learn more more about B-USEFUL in &lt;em&gt;About&lt;/em&gt; or at the  &lt;a href="https://b-useful.eu/"&gt;B-USEFUL project website&lt;/a&gt;.
-</t>
-  </si>
-  <si>
-    <t>&lt;h4&gt; How do I use this tool? &lt;/h4&gt;&lt;p&gt;&lt;li&gt;Select a case study region of interest from the dropdown or &lt;em&gt;Results&lt;/em&gt; tab of the navbar - you will be directed to the results.&lt;/li&gt;&lt;li&gt;use the &lt;em&gt;Explore&lt;/em&gt; tab to investigate the historical and projected changes in biodiversity for a range of indicators.&lt;/li&gt;&lt;li&gt;Use the  &lt;em&gt;Interactive tool&lt;/em&gt; tab to identify areas meeting your criteria.&lt;/li&gt;</t>
+    <t>&lt;dl&gt;
+&lt;dt&gt;Learn about the background of the work:&lt;/dt&gt;
+  &lt;dd&gt;Select&lt;em&gt;Background&lt;/em&gt; from the navabar at the top of page. Then scroll down through the descriptions of the projects context, objectives, data and scientific approach. &lt;/dd&gt;
+  &lt;dt&gt;Find the results:&lt;/dt&gt;
+  &lt;dd&gt;Select a case study region of interest from the dropdown or &lt;em&gt;Results&lt;/em&gt; tab of the navbar - you will be directed to the results.&lt;/dd&gt;
+&lt;details&gt;
+        &lt;summary&gt;Explore Biodiversity Spatial Patterns and Temporal Trends&lt;/summary&gt;
+&lt;p&gt;
+&lt;dt&gt;View animations of biodiversity development:&lt;/dt&gt;
+  &lt;dd&gt;Visiting &lt;em&gt;Results&lt;/em&gt;  automatically brings you to the &lt;em&gt;Biodiversity Development&lt;/em&gt; tab for the selected region. An animation of species richness development through time will automatically play. Other taxonomic and trait-based diversity indices can be selected from the sidebar. &lt;/dd&gt;
+&lt;dt&gt;Select years to compare biodiversity indices between:&lt;/dt&gt;
+  &lt;dd&gt;Switch from animations to side-by-side comparisons of specific years in the &lt;em&gt;Biodiversity Development sidebar&lt;/em&gt;. Pick years of interest from the &lt;em&gt;Year Selector&lt;/em&gt; input field.&lt;/dd&gt;
+&lt;dt&gt;View biodiversity trend:&lt;/dt&gt;
+  &lt;dd&gt;Toggle the &lt;em&gt;View biodiversity trend&lt;/em&gt; switch to show the biodiversity trend for the selected index across the whole period of data availability.&lt;/dd&gt;&lt;/p&gt;&lt;/details&gt;
+&lt;details&gt;
+        &lt;summary&gt;Use the Interactive Tool&lt;/summary&gt;
+&lt;p&gt;&lt;dt&gt;Apply biodiversity filters:&lt;/dt&gt;
+  &lt;dd&gt;&lt;ul&gt;Use the sidebar controls to:&lt;li&gt; Select which year of biodiversity results to apply filters to.&lt;/li&gt;
+&lt;li&gt;Filter areas of high or low biodiversity for different indices using the sliders.&lt;/li&gt;&lt;/ul&gt;&lt;/dd&gt;
+&lt;dt&gt;Apply spatial filters:&lt;/dt&gt;
+  &lt;dd&gt;Use the drawing tool to select an area of interest.
+&lt;/dd&gt;
+&lt;dt&gt;View Summary Statistics and Detailed Results:&lt;/dt&gt;
+  &lt;dd&gt; The biodiversity and spatial filters are combined and the tool provides a high-level statistical overview on the data as well as detailed outputs.
+&lt;/dd&gt;
+&lt;/p&gt;&lt;/details&gt;
+&lt;/dl&gt;</t>
   </si>
 </sst>
 </file>
@@ -568,15 +605,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFAC5F67-39A2-465C-88B9-4321F2EB8BB8}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="143.54296875" customWidth="1"/>
-    <col min="3" max="3" width="85.26953125" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="143.5703125" customWidth="1"/>
+    <col min="3" max="3" width="85.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -584,64 +621,72 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="88.5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="1" t="s">
+    <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A4" t="s">
-        <v>47</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
-      <c r="A6" t="s">
+    <row r="7" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A7" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
-      <c r="A8" t="s">
+    <row r="9" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="B9" s="1"/>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -652,13 +697,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98953C5C-C579-44AD-B9BC-A1CB08652AFC}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.86328125" customWidth="1"/>
-    <col min="2" max="2" width="92.86328125" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="92.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -666,7 +711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -674,7 +719,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -682,7 +727,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -690,7 +735,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="77.45" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" ht="77.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -698,7 +743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -706,12 +751,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -719,7 +764,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -735,13 +780,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{055D557F-35EA-4686-BF45-082A320EB9A3}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.7265625" customWidth="1"/>
-    <col min="2" max="2" width="79.54296875" customWidth="1"/>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="79.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -749,19 +794,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
     </row>
   </sheetData>
@@ -772,13 +817,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{815C4F49-50D2-4164-9FCA-37290B885711}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.26953125" customWidth="1"/>
-    <col min="2" max="2" width="72.1328125" customWidth="1"/>
+    <col min="1" max="1" width="20.28515625" customWidth="1"/>
+    <col min="2" max="2" width="72.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -786,31 +831,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" s="3"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" s="4"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="4"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" s="4"/>
     </row>
   </sheetData>
@@ -822,13 +867,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7534530D-A73A-4258-8656-ECA9512F2226}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.40625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="77.86328125" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="77.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -836,7 +881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -844,12 +889,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -862,12 +907,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24344193-A5DC-4C09-A7D0-962941565ADB}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="60.2265625" customWidth="1"/>
+    <col min="2" max="2" width="60.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -875,7 +920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -883,7 +928,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -891,7 +936,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -899,7 +944,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -907,7 +952,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -915,7 +960,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -923,7 +968,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -940,13 +985,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52622770-8B11-4F83-8FC4-BE5BFE84B716}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.58984375" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -954,7 +999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>

</xml_diff>

<commit_message>
Update tooltips and figure texts, improve layout across app
</commit_message>
<xml_diff>
--- a/data-raw/project_texts.xlsx
+++ b/data-raw/project_texts.xlsx
@@ -8,18 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neilm\Projects\b_useful\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FF5C0F-1624-4EC7-A5E8-F7570D3C0BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFFBEAE-1758-4A7C-A5E2-3CEE6DB8C7D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" activeTab="4" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="landing_page" sheetId="1" r:id="rId1"/>
-    <sheet name="story_map" sheetId="4" r:id="rId2"/>
-    <sheet name="themes" sheetId="2" r:id="rId3"/>
-    <sheet name="case_studies" sheetId="3" r:id="rId4"/>
-    <sheet name="fig_text" sheetId="5" r:id="rId5"/>
-    <sheet name="tooltips" sheetId="6" r:id="rId6"/>
-    <sheet name="sources" sheetId="7" r:id="rId7"/>
+    <sheet name="guidance" sheetId="8" r:id="rId2"/>
+    <sheet name="story_map" sheetId="4" r:id="rId3"/>
+    <sheet name="fig_text" sheetId="5" r:id="rId4"/>
+    <sheet name="tooltips" sheetId="6" r:id="rId5"/>
+    <sheet name="sources" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="57">
   <si>
     <t>text</t>
   </si>
@@ -107,15 +106,6 @@
   </si>
   <si>
     <t>time_comparison</t>
-  </si>
-  <si>
-    <t>biodiversity_animation</t>
-  </si>
-  <si>
-    <t>biodiversity_trend</t>
-  </si>
-  <si>
-    <t>Map of {taxon} {diversity_indicator} in the {ecoregion}.</t>
   </si>
   <si>
     <t>stakeholder_modal</t>
@@ -152,28 +142,10 @@
     <t>fdis</t>
   </si>
   <si>
-    <t>Functional evenness indices measure whether mean species traits are distributed regularly within the occupied trait space.</t>
-  </si>
-  <si>
-    <t>Functional Richness measures how much of the niche space is occupied by the species present.</t>
-  </si>
-  <si>
     <t>functional_diversity_indices</t>
   </si>
   <si>
     <t xml:space="preserve">Schleuter, Diana &amp; Daufresne, Martin &amp; Massol, François. (2010). A user's guide to functional diversity indices. Ecological Monographs. 80. 469-484. 10.2307/20787442. </t>
-  </si>
-  <si>
-    <t>Functional divergence measures the variance of the species’ functions and the position of their clusters in trait space. High values indicate that the dominant species have extreme traits.</t>
-  </si>
-  <si>
-    <t>Function dispersion measures how far species are, on average, from the community average traits. High values indicate an assemblage where species are generally quite different and where there are many ecological roles.</t>
-  </si>
-  <si>
-    <t>Species Richness is the number of species that are present in a given area.</t>
-  </si>
-  <si>
-    <t>Shannon Index measures the proportional abundance of species in an assemblage. For a given number of species, an assemblage with higher evenness will have a higher shannon index.</t>
   </si>
   <si>
     <t>Relative abundance of different species within a community or ecosystem.</t>
@@ -231,30 +203,111 @@
 &lt;/p&gt;&lt;/details&gt;
 &lt;/dl&gt;</t>
   </si>
+  <si>
+    <t>interactive_tool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;h5&gt;Overview&lt;/h5&gt;
+    &lt;p&gt;
+      This tool allows you to identify and explore areas of biodiversity importance
+      by combining biodiversity filters with a user-defined spatial selection.
+    &lt;/p&gt;
+    &lt;h5&gt;Workflow&lt;/h5&gt;
+    &lt;ol&gt;
+      &lt;li&gt;
+        &lt;strong&gt;Configure biodiversity filters&lt;/strong&gt;&lt;br&gt;
+        Select a biodiversity year and adjust the percentile ranges for one or more
+        biodiversity metrics. Only locations meeting all selected criteria will be retained.
+      &lt;/li&gt;
+      &lt;li&gt;
+        &lt;strong&gt;Define an area of interest&lt;/strong&gt;&lt;br&gt;
+        Use the drawing tools on the map to create one or more polygons representing
+        your area of interest.
+      &lt;/li&gt;
+      &lt;li&gt;
+        &lt;strong&gt;Review biodiversity statistics&lt;/strong&gt;&lt;br&gt;
+        Summary statistics and detailed information are generated for locations that
+        satisfy both the biodiversity and spatial filters.
+      &lt;/li&gt;
+      &lt;li&gt;
+        &lt;strong&gt;Explore future overlays&lt;/strong&gt;&lt;br&gt;
+        Future versions of the tool will support the visualization of human activities
+        within the selected area.
+      &lt;/li&gt;
+    &lt;/ol&gt;
+    &lt;h5&gt;How filtering works&lt;/h5&gt;
+    &lt;p&gt;
+      Biodiversity and spatial filters are applied together. A location must:
+    &lt;/p&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Fall within the user-defined spatial selection; and&lt;/li&gt;
+      &lt;li&gt;Meet all selected biodiversity filter criteria.&lt;/li&gt;
+    &lt;/ul&gt;
+    &lt;div class='alert alert-info'&gt;
+      &lt;strong&gt;Tip:&lt;/strong&gt; Start with broad biodiversity filter ranges and a large
+      spatial selection, then progressively narrow your criteria to identify
+      biodiversity hotspots or areas with specific ecological characteristics.
+    &lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>animation_trend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;strong&gt;Left panel&lt;/strong&gt; Animation of development of {taxon} {diversity_indicator} in the {ecoregion}.&lt;br&gt;
+&lt;strong&gt;Right panel&lt;/strong&gt; Linear trend in {taxon} {diversity_indicator} in the {ecoregion} between {yr_summary[1]} and {yr_summary[6]}.
+</t>
+  </si>
+  <si>
+    <t>Spatial patterns
+of  {taxon} {diversity_indicator} in the {ecoregion}. &lt;br&gt;The indicators are
+based on model predictions for the selected years: {years}.</t>
+  </si>
+  <si>
+    <t>diversity_filters</t>
+  </si>
+  <si>
+    <t>Filtered spatial patterns
+of  {taxon} {diversity_indicator} in the {ecoregion}. Only locations that meet all user defined selection criteria are retained: &lt;br&gt;
+&lt;strong&gt;Species Richness Percentiles:&lt;/strong&gt; {rich_pct};
+&lt;strong&gt;Evenness Percentiles:&lt;/strong&gt; {eve_pct};
+&lt;strong&gt;Shannon Index Percentiles:&lt;/strong&gt; {shannon_pct};
+&lt;strong&gt;Functional Richness Percentiles:&lt;/strong&gt; {fric_pct};
+&lt;strong&gt;Functional Evenness Percentiles:&lt;/strong&gt; {feve_pct};
+&lt;strong&gt;Functional Dispersion Percentiles:&lt;/strong&gt; {fdis_pct};
+&lt;strong&gt;Functional Divergence Percentiles:&lt;/strong&gt; {fdiv_pct}.
+&lt;br&gt;The indicators are
+based on model predictions for the selected year: {yr}.</t>
+  </si>
+  <si>
+    <t>Measures the proportional abundance of species in an assemblage. For a given number of species, an assemblage with higher evenness will have a higher shannon index.</t>
+  </si>
+  <si>
+    <t>Number of species that are present in a given area.</t>
+  </si>
+  <si>
+    <t>Volume of functional trait space occupied.</t>
+  </si>
+  <si>
+    <t>Measures whether mean species traits are distributed regularly within the occupied trait space.</t>
+  </si>
+  <si>
+    <t>Variance of the species’ functions and the position of their clusters in trait space. High values indicate that the dominant species have extreme traits.</t>
+  </si>
+  <si>
+    <t>How far species are, on average, from the community average traits. High values indicate an assemblage where species are generally quite different and where there are many ecological roles.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF210384"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="4"/>
-      <color rgb="FF210384"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -277,19 +330,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -606,14 +650,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFAC5F67-39A2-465C-88B9-4321F2EB8BB8}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="143.5703125" customWidth="1"/>
-    <col min="3" max="3" width="85.28515625" customWidth="1"/>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="143.54296875" customWidth="1"/>
+    <col min="3" max="3" width="85.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -621,39 +665,39 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="88.5" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="59" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -661,7 +705,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -669,7 +713,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -677,15 +721,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
       <c r="B10" s="1"/>
     </row>
   </sheetData>
@@ -695,15 +739,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98953C5C-C579-44AD-B9BC-A1CB08652AFC}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCDFC4F4-DA9B-4676-B4E9-27438403FC6D}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" customWidth="1"/>
-    <col min="2" max="2" width="92.85546875" customWidth="1"/>
+    <col min="1" max="1" width="14.08984375" customWidth="1"/>
+    <col min="2" max="2" width="110.40625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -711,65 +755,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="77.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
+        <v>44</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -778,15 +769,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{055D557F-35EA-4686-BF45-082A320EB9A3}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98953C5C-C579-44AD-B9BC-A1CB08652AFC}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="79.5703125" customWidth="1"/>
+    <col min="1" max="1" width="26.86328125" customWidth="1"/>
+    <col min="2" max="2" width="92.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -794,20 +785,66 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B2" s="1"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B3" s="2"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B5" s="2"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B6" s="1"/>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="77.45" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -815,15 +852,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{815C4F49-50D2-4164-9FCA-37290B885711}">
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7534530D-A73A-4258-8656-ECA9512F2226}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" customWidth="1"/>
-    <col min="2" max="2" width="72.140625" customWidth="1"/>
+    <col min="1" max="1" width="19.40625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="77.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -831,72 +868,28 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B2" s="1"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B5" s="1"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B8" s="3"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B9" s="4"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B10" s="4"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B11" s="4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7534530D-A73A-4258-8656-ECA9512F2226}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="77.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="73.75" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="177" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>49</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -904,15 +897,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24344193-A5DC-4C09-A7D0-962941565ADB}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="60.28515625" customWidth="1"/>
+    <col min="2" max="2" width="60.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -920,60 +913,60 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
         <v>30</v>
       </c>
-      <c r="B2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
         <v>31</v>
       </c>
-      <c r="B3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
         <v>32</v>
       </c>
-      <c r="B4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A8" t="s">
         <v>33</v>
       </c>
-      <c r="B5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>36</v>
-      </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -982,16 +975,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52622770-8B11-4F83-8FC4-BE5BFE84B716}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+    <col min="1" max="1" width="25.54296875" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -999,12 +992,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add download tab with links to zipfiles
</commit_message>
<xml_diff>
--- a/data-raw/project_texts.xlsx
+++ b/data-raw/project_texts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neilm\Projects\b_useful\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFFBEAE-1758-4A7C-A5E2-3CEE6DB8C7D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61BA3F59-8C53-4346-B96A-703675A8BD12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" activeTab="4" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" activeTab="5" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="landing_page" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="story_map" sheetId="4" r:id="rId3"/>
     <sheet name="fig_text" sheetId="5" r:id="rId4"/>
     <sheet name="tooltips" sheetId="6" r:id="rId5"/>
-    <sheet name="sources" sheetId="7" r:id="rId6"/>
+    <sheet name="downloads" sheetId="9" r:id="rId6"/>
+    <sheet name="sources" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="67">
   <si>
     <t>text</t>
   </si>
@@ -295,6 +296,61 @@
   </si>
   <si>
     <t>How far species are, on average, from the community average traits. High values indicate an assemblage where species are generally quite different and where there are many ecological roles.</t>
+  </si>
+  <si>
+    <t>introduction</t>
+  </si>
+  <si>
+    <t>ce_med</t>
+  </si>
+  <si>
+    <t>iceland</t>
+  </si>
+  <si>
+    <t>ne_atlantic</t>
+  </si>
+  <si>
+    <t>wmed</t>
+  </si>
+  <si>
+    <t>The data bundle consists of the following files&lt;ul&gt;
+&lt;li&gt;A Disclaimer&lt;/li&gt;
+&lt;li&gt;Probabilities of species occurrences&lt;/li&gt;
+&lt;li&gt;Predicted species abundances&lt;/li&gt;
+&lt;li&gt;Species Traits&lt;/li&gt;
+&lt;li&gt;Biodiversity Indices derived from modelled species occurrences and trait data&lt;/li&gt;
+&lt;li&gt;Model Diagnostics&lt;/li&gt;</t>
+  </si>
+  <si>
+    <t>The data bundle consists of the following files&lt;ul&gt;
+&lt;li&gt;A Disclaimer&lt;/li&gt;
+&lt;li&gt;Probabilities of species occurrences&lt;/li&gt;
+&lt;li&gt;Predicted species biomass&lt;/li&gt;
+&lt;li&gt;Species Traits&lt;/li&gt;
+&lt;li&gt;Biodiversity Indices derived from modelled species occurrences and trait data&lt;/li&gt;
+&lt;li&gt;Model Diagnostics&lt;/li&gt;</t>
+  </si>
+  <si>
+    <t>The data bundle consists of the following files&lt;ul&gt;
+&lt;li&gt;A Disclaimer&lt;/li&gt;
+&lt;li&gt;Probabilities of species occurrences&lt;/li&gt;
+&lt;li&gt;Predicted species abundance&lt;/li&gt;
+&lt;li&gt;Species Traits&lt;/li&gt;
+&lt;li&gt;Biodiversity Indices derived from modelled species occurrences and trait data&lt;/li&gt;
+&lt;li&gt;Model Diagnostics&lt;/li&gt;</t>
+  </si>
+  <si>
+    <t>The data bundle consists of the following files&lt;ul&gt;
+&lt;li&gt;A Disclaimer&lt;/li&gt;
+&lt;li&gt;Probabilities of species occurrences&lt;/li&gt;
+&lt;li&gt;Species Traits&lt;/li&gt;
+&lt;li&gt;Biodiversity Indices derived from modelled species occurrences and trait data&lt;/li&gt;
+&lt;li&gt;Model Diagnostics&lt;/li&gt;</t>
+  </si>
+  <si>
+    <t>B-USEFUL's model outputs are available the &lt;a hfef="https://creativecommons.org/licenses/by/4.0/ "&gt; CC BY 4.0 license&lt;/a&gt;&lt;br&gt;
+Please feel free to download and use the data, providing attribution to the authors.&lt;br&gt;&lt;br&gt;
+The data is available as a zipfile bundle per model. Select from the models to see the available data and access the download link.</t>
   </si>
 </sst>
 </file>
@@ -976,6 +1032,67 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D71172A-305B-48CD-890B-1E71821EDF52}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <cols>
+    <col min="2" max="2" width="95.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="73.75" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="88.5" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52622770-8B11-4F83-8FC4-BE5BFE84B716}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>

</xml_diff>

<commit_message>
Fix legend labels, facet title sizing, interactive tool figure, metric names in tables
</commit_message>
<xml_diff>
--- a/data-raw/project_texts.xlsx
+++ b/data-raw/project_texts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neilm\Projects\b_useful\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61BA3F59-8C53-4346-B96A-703675A8BD12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4A866A-7BA4-4424-8217-47BC6DFF66F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" activeTab="5" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" firstSheet="1" activeTab="3" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="landing_page" sheetId="1" r:id="rId1"/>
@@ -267,19 +267,6 @@
     <t>diversity_filters</t>
   </si>
   <si>
-    <t>Filtered spatial patterns
-of  {taxon} {diversity_indicator} in the {ecoregion}. Only locations that meet all user defined selection criteria are retained: &lt;br&gt;
-&lt;strong&gt;Species Richness Percentiles:&lt;/strong&gt; {rich_pct};
-&lt;strong&gt;Evenness Percentiles:&lt;/strong&gt; {eve_pct};
-&lt;strong&gt;Shannon Index Percentiles:&lt;/strong&gt; {shannon_pct};
-&lt;strong&gt;Functional Richness Percentiles:&lt;/strong&gt; {fric_pct};
-&lt;strong&gt;Functional Evenness Percentiles:&lt;/strong&gt; {feve_pct};
-&lt;strong&gt;Functional Dispersion Percentiles:&lt;/strong&gt; {fdis_pct};
-&lt;strong&gt;Functional Divergence Percentiles:&lt;/strong&gt; {fdiv_pct}.
-&lt;br&gt;The indicators are
-based on model predictions for the selected year: {yr}.</t>
-  </si>
-  <si>
     <t>Measures the proportional abundance of species in an assemblage. For a given number of species, an assemblage with higher evenness will have a higher shannon index.</t>
   </si>
   <si>
@@ -351,6 +338,19 @@
     <t>B-USEFUL's model outputs are available the &lt;a hfef="https://creativecommons.org/licenses/by/4.0/ "&gt; CC BY 4.0 license&lt;/a&gt;&lt;br&gt;
 Please feel free to download and use the data, providing attribution to the authors.&lt;br&gt;&lt;br&gt;
 The data is available as a zipfile bundle per model. Select from the models to see the available data and access the download link.</t>
+  </si>
+  <si>
+    <t>Filtered spatial patterns
+of  {taxon} {diversity_indicator} in the {ecoregion}. Only locations that meet all user defined selection criteria are retained: &lt;br&gt;
+&lt;strong&gt;Species Richness Percentiles:&lt;/strong&gt; {rich_pct};
+&lt;strong&gt;Evenness Percentiles:&lt;/strong&gt; {eve_pct};&lt;br&gt;
+&lt;strong&gt;Shannon Index Percentiles:&lt;/strong&gt; {shannon_pct};
+&lt;strong&gt;Functional Richness Percentiles:&lt;/strong&gt; {fric_pct};&lt;br&gt;
+&lt;strong&gt;Functional Evenness Percentiles:&lt;/strong&gt; {feve_pct};
+&lt;strong&gt;Functional Dispersion Percentiles:&lt;/strong&gt; {fdis_pct};&lt;br&gt;
+&lt;strong&gt;Functional Divergence Percentiles:&lt;/strong&gt; {fdiv_pct}.
+&lt;br&gt;The indicators are
+based on model predictions for the selected year: {yr}.</t>
   </si>
 </sst>
 </file>
@@ -945,7 +945,7 @@
         <v>49</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -974,7 +974,7 @@
         <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.75">
@@ -990,7 +990,7 @@
         <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.75">
@@ -998,7 +998,7 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.75">
@@ -1006,7 +1006,7 @@
         <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.75">
@@ -1014,7 +1014,7 @@
         <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.75">
@@ -1022,7 +1022,7 @@
         <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1049,42 +1049,42 @@
     </row>
     <row r="2" spans="1:2" ht="73.75" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="88.5" x14ac:dyDescent="0.75">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>